<commit_message>
Reorder consolidated turnover sections
</commit_message>
<xml_diff>
--- a/output/spreadsheet/pyg_consolidado_2026.xlsx
+++ b/output/spreadsheet/pyg_consolidado_2026.xlsx
@@ -712,7 +712,7 @@
     <row r="3" ht="12" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Actualizado: 04/04/2026 12:00 h</t>
+          <t>Actualizado: 04/04/2026 12:10 h</t>
         </is>
       </c>
     </row>
@@ -725,51 +725,51 @@
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="6">
-        <f>D5+D8+D11</f>
+        <f>D5+D10+D11</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>E5+E8+E11</f>
+        <f>E5+E10+E11</f>
         <v/>
       </c>
       <c r="F4" s="6">
-        <f>F5+F8+F11</f>
+        <f>F5+F10+F11</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>G5+G8+G11</f>
+        <f>G5+G10+G11</f>
         <v/>
       </c>
       <c r="H4" s="6">
-        <f>H5+H8+H11</f>
+        <f>H5+H10+H11</f>
         <v/>
       </c>
       <c r="I4" s="6">
-        <f>I5+I8+I11</f>
+        <f>I5+I10+I11</f>
         <v/>
       </c>
       <c r="J4" s="6">
-        <f>J5+J8+J11</f>
+        <f>J5+J10+J11</f>
         <v/>
       </c>
       <c r="K4" s="6">
-        <f>K5+K8+K11</f>
+        <f>K5+K10+K11</f>
         <v/>
       </c>
       <c r="L4" s="6">
-        <f>L5+L8+L11</f>
+        <f>L5+L10+L11</f>
         <v/>
       </c>
       <c r="M4" s="6">
-        <f>M5+M8+M11</f>
+        <f>M5+M10+M11</f>
         <v/>
       </c>
       <c r="N4" s="6">
-        <f>N5+N8+N11</f>
+        <f>N5+N10+N11</f>
         <v/>
       </c>
       <c r="O4" s="6">
-        <f>O5+O8+O11</f>
+        <f>O5+O10+O11</f>
         <v/>
       </c>
       <c r="P4" s="7">
@@ -786,51 +786,51 @@
       <c r="B5" s="9" t="n"/>
       <c r="C5" s="9" t="n"/>
       <c r="D5" s="10">
-        <f>D6+D7+D9+D10</f>
+        <f>D6+D7+D8+D9</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>E6+E7+E9+E10</f>
+        <f>E6+E7+E8+E9</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>F6+F7+F9+F10</f>
+        <f>F6+F7+F8+F9</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>G6+G7+G9+G10</f>
+        <f>G6+G7+G8+G9</f>
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>H6+H7+H9+H10</f>
+        <f>H6+H7+H8+H9</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>I6+I7+I9+I10</f>
+        <f>I6+I7+I8+I9</f>
         <v/>
       </c>
       <c r="J5" s="10">
-        <f>J6+J7+J9+J10</f>
+        <f>J6+J7+J8+J9</f>
         <v/>
       </c>
       <c r="K5" s="10">
-        <f>K6+K7+K9+K10</f>
+        <f>K6+K7+K8+K9</f>
         <v/>
       </c>
       <c r="L5" s="10">
-        <f>L6+L7+L9+L10</f>
+        <f>L6+L7+L8+L9</f>
         <v/>
       </c>
       <c r="M5" s="10">
-        <f>M6+M7+M9+M10</f>
+        <f>M6+M7+M8+M9</f>
         <v/>
       </c>
       <c r="N5" s="10">
-        <f>N6+N7+N9+N10</f>
+        <f>N6+N7+N8+N9</f>
         <v/>
       </c>
       <c r="O5" s="10">
-        <f>O6+O7+O9+O10</f>
+        <f>O6+O7+O8+O9</f>
         <v/>
       </c>
       <c r="P5" s="11">
@@ -957,62 +957,60 @@
       </c>
     </row>
     <row r="8" ht="12" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>Services</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="10">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,D$1,'i-sl'!$B:$B,"services_ext")</f>
-        <v/>
-      </c>
-      <c r="E8" s="10">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,E$1,'i-sl'!$B:$B,"services_ext")</f>
-        <v/>
-      </c>
-      <c r="F8" s="10">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,F$1,'i-sl'!$B:$B,"services_ext")</f>
-        <v/>
-      </c>
-      <c r="G8" s="10">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,G$1,'i-sl'!$B:$B,"services_ext")</f>
-        <v/>
-      </c>
-      <c r="H8" s="10">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,H$1,'i-sl'!$B:$B,"services_ext")</f>
-        <v/>
-      </c>
-      <c r="I8" s="10">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,I$1,'i-sl'!$B:$B,"services_ext")</f>
-        <v/>
-      </c>
-      <c r="J8" s="10">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,J$1,'i-sl'!$B:$B,"services_ext")</f>
-        <v/>
-      </c>
-      <c r="K8" s="10">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,K$1,'i-sl'!$B:$B,"services_ext")</f>
-        <v/>
-      </c>
-      <c r="L8" s="10">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,L$1,'i-sl'!$B:$B,"services_ext")</f>
-        <v/>
-      </c>
-      <c r="M8" s="10">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,M$1,'i-sl'!$B:$B,"services_ext")</f>
-        <v/>
-      </c>
-      <c r="N8" s="10">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,N$1,'i-sl'!$B:$B,"services_ext")</f>
-        <v/>
-      </c>
-      <c r="O8" s="10">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,O$1,'i-sl'!$B:$B,"services_ext")</f>
-        <v/>
-      </c>
-      <c r="P8" s="11">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Rappels</t>
+        </is>
+      </c>
+      <c r="D8" s="13">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,D$1,'i-sl'!$B:$B,"rappels")</f>
+        <v/>
+      </c>
+      <c r="E8" s="13">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,E$1,'i-sl'!$B:$B,"rappels")</f>
+        <v/>
+      </c>
+      <c r="F8" s="13">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,F$1,'i-sl'!$B:$B,"rappels")</f>
+        <v/>
+      </c>
+      <c r="G8" s="13">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,G$1,'i-sl'!$B:$B,"rappels")</f>
+        <v/>
+      </c>
+      <c r="H8" s="13">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,H$1,'i-sl'!$B:$B,"rappels")</f>
+        <v/>
+      </c>
+      <c r="I8" s="13">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,I$1,'i-sl'!$B:$B,"rappels")</f>
+        <v/>
+      </c>
+      <c r="J8" s="13">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,J$1,'i-sl'!$B:$B,"rappels")</f>
+        <v/>
+      </c>
+      <c r="K8" s="13">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,K$1,'i-sl'!$B:$B,"rappels")</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,L$1,'i-sl'!$B:$B,"rappels")</f>
+        <v/>
+      </c>
+      <c r="M8" s="13">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,M$1,'i-sl'!$B:$B,"rappels")</f>
+        <v/>
+      </c>
+      <c r="N8" s="13">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,N$1,'i-sl'!$B:$B,"rappels")</f>
+        <v/>
+      </c>
+      <c r="O8" s="13">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,O$1,'i-sl'!$B:$B,"rappels")</f>
+        <v/>
+      </c>
+      <c r="P8" s="14">
         <f>SUM(D8:O8)</f>
         <v/>
       </c>
@@ -1020,55 +1018,55 @@
     <row r="9" ht="12" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Rappels</t>
+          <t>Supplies</t>
         </is>
       </c>
       <c r="D9" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,D$1,'i-sl'!$B:$B,"rappels")</f>
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,D$1,'i-sl'!$B:$B,"supplies")</f>
         <v/>
       </c>
       <c r="E9" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,E$1,'i-sl'!$B:$B,"rappels")</f>
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,E$1,'i-sl'!$B:$B,"supplies")</f>
         <v/>
       </c>
       <c r="F9" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,F$1,'i-sl'!$B:$B,"rappels")</f>
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,F$1,'i-sl'!$B:$B,"supplies")</f>
         <v/>
       </c>
       <c r="G9" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,G$1,'i-sl'!$B:$B,"rappels")</f>
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,G$1,'i-sl'!$B:$B,"supplies")</f>
         <v/>
       </c>
       <c r="H9" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,H$1,'i-sl'!$B:$B,"rappels")</f>
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,H$1,'i-sl'!$B:$B,"supplies")</f>
         <v/>
       </c>
       <c r="I9" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,I$1,'i-sl'!$B:$B,"rappels")</f>
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,I$1,'i-sl'!$B:$B,"supplies")</f>
         <v/>
       </c>
       <c r="J9" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,J$1,'i-sl'!$B:$B,"rappels")</f>
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,J$1,'i-sl'!$B:$B,"supplies")</f>
         <v/>
       </c>
       <c r="K9" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,K$1,'i-sl'!$B:$B,"rappels")</f>
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,K$1,'i-sl'!$B:$B,"supplies")</f>
         <v/>
       </c>
       <c r="L9" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,L$1,'i-sl'!$B:$B,"rappels")</f>
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,L$1,'i-sl'!$B:$B,"supplies")</f>
         <v/>
       </c>
       <c r="M9" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,M$1,'i-sl'!$B:$B,"rappels")</f>
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,M$1,'i-sl'!$B:$B,"supplies")</f>
         <v/>
       </c>
       <c r="N9" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,N$1,'i-sl'!$B:$B,"rappels")</f>
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,N$1,'i-sl'!$B:$B,"supplies")</f>
         <v/>
       </c>
       <c r="O9" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,O$1,'i-sl'!$B:$B,"rappels")</f>
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,O$1,'i-sl'!$B:$B,"supplies")</f>
         <v/>
       </c>
       <c r="P9" s="14">
@@ -1077,60 +1075,62 @@
       </c>
     </row>
     <row r="10" ht="12" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Supplies</t>
-        </is>
-      </c>
-      <c r="D10" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,D$1,'i-sl'!$B:$B,"supplies")</f>
-        <v/>
-      </c>
-      <c r="E10" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,E$1,'i-sl'!$B:$B,"supplies")</f>
-        <v/>
-      </c>
-      <c r="F10" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,F$1,'i-sl'!$B:$B,"supplies")</f>
-        <v/>
-      </c>
-      <c r="G10" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,G$1,'i-sl'!$B:$B,"supplies")</f>
-        <v/>
-      </c>
-      <c r="H10" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,H$1,'i-sl'!$B:$B,"supplies")</f>
-        <v/>
-      </c>
-      <c r="I10" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,I$1,'i-sl'!$B:$B,"supplies")</f>
-        <v/>
-      </c>
-      <c r="J10" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,J$1,'i-sl'!$B:$B,"supplies")</f>
-        <v/>
-      </c>
-      <c r="K10" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,K$1,'i-sl'!$B:$B,"supplies")</f>
-        <v/>
-      </c>
-      <c r="L10" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,L$1,'i-sl'!$B:$B,"supplies")</f>
-        <v/>
-      </c>
-      <c r="M10" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,M$1,'i-sl'!$B:$B,"supplies")</f>
-        <v/>
-      </c>
-      <c r="N10" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,N$1,'i-sl'!$B:$B,"supplies")</f>
-        <v/>
-      </c>
-      <c r="O10" s="13">
-        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,O$1,'i-sl'!$B:$B,"supplies")</f>
-        <v/>
-      </c>
-      <c r="P10" s="14">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n"/>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="10">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,D$1,'i-sl'!$B:$B,"services_ext")</f>
+        <v/>
+      </c>
+      <c r="E10" s="10">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,E$1,'i-sl'!$B:$B,"services_ext")</f>
+        <v/>
+      </c>
+      <c r="F10" s="10">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,F$1,'i-sl'!$B:$B,"services_ext")</f>
+        <v/>
+      </c>
+      <c r="G10" s="10">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,G$1,'i-sl'!$B:$B,"services_ext")</f>
+        <v/>
+      </c>
+      <c r="H10" s="10">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,H$1,'i-sl'!$B:$B,"services_ext")</f>
+        <v/>
+      </c>
+      <c r="I10" s="10">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,I$1,'i-sl'!$B:$B,"services_ext")</f>
+        <v/>
+      </c>
+      <c r="J10" s="10">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,J$1,'i-sl'!$B:$B,"services_ext")</f>
+        <v/>
+      </c>
+      <c r="K10" s="10">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,K$1,'i-sl'!$B:$B,"services_ext")</f>
+        <v/>
+      </c>
+      <c r="L10" s="10">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,L$1,'i-sl'!$B:$B,"services_ext")</f>
+        <v/>
+      </c>
+      <c r="M10" s="10">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,M$1,'i-sl'!$B:$B,"services_ext")</f>
+        <v/>
+      </c>
+      <c r="N10" s="10">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,N$1,'i-sl'!$B:$B,"services_ext")</f>
+        <v/>
+      </c>
+      <c r="O10" s="10">
+        <f>SUMIFS('i-sl'!$C:$C,'i-sl'!$A:$A,O$1,'i-sl'!$B:$B,"services_ext")</f>
+        <v/>
+      </c>
+      <c r="P10" s="11">
         <f>SUM(D10:O10)</f>
         <v/>
       </c>
@@ -4601,28 +4601,28 @@
       </c>
     </row>
     <row r="8" ht="12" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>Services</t>
-        </is>
-      </c>
-      <c r="B8" s="10">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Rappels</t>
+        </is>
+      </c>
+      <c r="B8" s="13">
         <f>SUM('P&amp;G-CONSOLIDADO'!D8:F8)</f>
         <v/>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="13">
         <f>SUM('P&amp;G-CONSOLIDADO'!G8:I8)</f>
         <v/>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="13">
         <f>SUM('P&amp;G-CONSOLIDADO'!J8:L8)</f>
         <v/>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="13">
         <f>SUM('P&amp;G-CONSOLIDADO'!M8:O8)</f>
         <v/>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="14">
         <f>'P&amp;G-CONSOLIDADO'!P8</f>
         <v/>
       </c>
@@ -4630,7 +4630,7 @@
     <row r="9" ht="12" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Rappels</t>
+          <t>Supplies</t>
         </is>
       </c>
       <c r="B9" s="13">
@@ -4655,28 +4655,28 @@
       </c>
     </row>
     <row r="10" ht="12" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Supplies</t>
-        </is>
-      </c>
-      <c r="B10" s="13">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="B10" s="10">
         <f>SUM('P&amp;G-CONSOLIDADO'!D10:F10)</f>
         <v/>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="10">
         <f>SUM('P&amp;G-CONSOLIDADO'!G10:I10)</f>
         <v/>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="10">
         <f>SUM('P&amp;G-CONSOLIDADO'!J10:L10)</f>
         <v/>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="10">
         <f>SUM('P&amp;G-CONSOLIDADO'!M10:O10)</f>
         <v/>
       </c>
-      <c r="F10" s="14">
+      <c r="F10" s="11">
         <f>'P&amp;G-CONSOLIDADO'!P10</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add Contasimple invoice parser
</commit_message>
<xml_diff>
--- a/output/spreadsheet/pyg_consolidado_2026.xlsx
+++ b/output/spreadsheet/pyg_consolidado_2026.xlsx
@@ -712,7 +712,7 @@
     <row r="3" ht="12" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Actualizado: 04/04/2026 12:10 h</t>
+          <t>Actualizado: 10/04/2026 11:48 h</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2835,7 +2835,7 @@
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>1222.08</v>
+        <v>2753.58</v>
       </c>
     </row>
     <row r="33" ht="12" customHeight="1">
@@ -2850,7 +2850,7 @@
         </is>
       </c>
       <c r="C33" s="23" t="n">
-        <v>1915.94</v>
+        <v>16086.79</v>
       </c>
     </row>
     <row r="34" ht="12" customHeight="1">
@@ -2895,7 +2895,7 @@
         </is>
       </c>
       <c r="C36" s="23" t="n">
-        <v>15609.96</v>
+        <v>16887.89</v>
       </c>
     </row>
     <row r="37" ht="12" customHeight="1">
@@ -2936,11 +2936,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>shopify</t>
+          <t>services_ext</t>
         </is>
       </c>
       <c r="C39" s="23" t="n">
-        <v>153533.23</v>
+        <v>595.59</v>
       </c>
     </row>
     <row r="40" ht="12" customHeight="1">
@@ -2951,11 +2951,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>staff</t>
+          <t>shopify</t>
         </is>
       </c>
       <c r="C40" s="23" t="n">
-        <v>15349.42</v>
+        <v>153533.23</v>
       </c>
     </row>
     <row r="41" ht="12" customHeight="1">
@@ -2966,11 +2966,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>supplies</t>
+          <t>staff</t>
         </is>
       </c>
       <c r="C41" s="23" t="n">
-        <v>-585.21</v>
+        <v>15349.42</v>
       </c>
     </row>
     <row r="42" ht="12" customHeight="1">
@@ -2981,26 +2981,26 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>technology</t>
+          <t>supplies</t>
         </is>
       </c>
       <c r="C42" s="23" t="n">
-        <v>5290.69</v>
+        <v>-585.21</v>
       </c>
     </row>
     <row r="43" ht="12" customHeight="1">
       <c r="A43" t="inlineStr">
         <is>
-          <t>202604</t>
+          <t>202603</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>payment_fees</t>
+          <t>technology</t>
         </is>
       </c>
       <c r="C43" s="23" t="n">
-        <v>434.69</v>
+        <v>5355.88</v>
       </c>
     </row>
     <row r="44" ht="12" customHeight="1">
@@ -3011,11 +3011,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>shopify</t>
+          <t>administration</t>
         </is>
       </c>
       <c r="C44" s="23" t="n">
-        <v>25715.9</v>
+        <v>823.08</v>
       </c>
     </row>
     <row r="45" ht="12" customHeight="1">
@@ -3026,11 +3026,41 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
+          <t>payment_fees</t>
+        </is>
+      </c>
+      <c r="C45" s="23" t="n">
+        <v>948.47</v>
+      </c>
+    </row>
+    <row r="46" ht="12" customHeight="1">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>202604</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="C46" s="23" t="n">
+        <v>54823.58</v>
+      </c>
+    </row>
+    <row r="47" ht="12" customHeight="1">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>202604</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>technology</t>
         </is>
       </c>
-      <c r="C45" s="23" t="n">
-        <v>163.48</v>
+      <c r="C47" s="23" t="n">
+        <v>163.1</v>
       </c>
     </row>
   </sheetData>
@@ -3231,7 +3261,7 @@
         </is>
       </c>
       <c r="C12" s="23" t="n">
-        <v>185.17</v>
+        <v>254.17</v>
       </c>
     </row>
     <row r="13" ht="12" customHeight="1">
@@ -3321,7 +3351,7 @@
         </is>
       </c>
       <c r="C18" s="23" t="n">
-        <v>185.17</v>
+        <v>1035.17</v>
       </c>
     </row>
     <row r="19" ht="12" customHeight="1">
@@ -3336,7 +3366,7 @@
         </is>
       </c>
       <c r="C19" s="23" t="n">
-        <v>67.65000000000001</v>
+        <v>284.82</v>
       </c>
     </row>
     <row r="20" ht="12" customHeight="1">
@@ -3351,7 +3381,7 @@
         </is>
       </c>
       <c r="C20" s="23" t="n">
-        <v>35.85</v>
+        <v>117.4</v>
       </c>
     </row>
     <row r="21" ht="12" customHeight="1">
@@ -3366,7 +3396,7 @@
         </is>
       </c>
       <c r="C21" s="23" t="n">
-        <v>1333.46</v>
+        <v>5572.05</v>
       </c>
     </row>
     <row r="22" ht="12" customHeight="1">
@@ -3867,7 +3897,7 @@
         </is>
       </c>
       <c r="C16" s="23" t="n">
-        <v>1150</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="17" ht="12" customHeight="1">
@@ -3882,7 +3912,7 @@
         </is>
       </c>
       <c r="C17" s="23" t="n">
-        <v>58.35</v>
+        <v>67.3</v>
       </c>
     </row>
     <row r="18" ht="12" customHeight="1">
@@ -3897,7 +3927,7 @@
         </is>
       </c>
       <c r="C18" s="23" t="n">
-        <v>43.42</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" ht="12" customHeight="1">
@@ -3912,7 +3942,7 @@
         </is>
       </c>
       <c r="C19" s="23" t="n">
-        <v>1645.88</v>
+        <v>4493.94</v>
       </c>
     </row>
     <row r="20" ht="12" customHeight="1">
@@ -4173,7 +4203,7 @@
         </is>
       </c>
       <c r="C8" s="24" t="n">
-        <v>0.87253</v>
+        <v>0.87053</v>
       </c>
     </row>
     <row r="9" ht="12" customHeight="1">
@@ -4188,7 +4218,7 @@
         </is>
       </c>
       <c r="C9" s="24" t="n">
-        <v>1.1525</v>
+        <v>1.1685</v>
       </c>
     </row>
     <row r="10" ht="12" customHeight="1">
@@ -4203,7 +4233,7 @@
         </is>
       </c>
       <c r="C10" s="24" t="n">
-        <v>0.87253</v>
+        <v>0.87053</v>
       </c>
     </row>
     <row r="11" ht="12" customHeight="1">
@@ -4218,7 +4248,7 @@
         </is>
       </c>
       <c r="C11" s="24" t="n">
-        <v>1.1525</v>
+        <v>1.1685</v>
       </c>
     </row>
     <row r="12" ht="12" customHeight="1">
@@ -4233,7 +4263,7 @@
         </is>
       </c>
       <c r="C12" s="24" t="n">
-        <v>0.87253</v>
+        <v>0.87053</v>
       </c>
     </row>
     <row r="13" ht="12" customHeight="1">
@@ -4248,7 +4278,7 @@
         </is>
       </c>
       <c r="C13" s="24" t="n">
-        <v>1.1525</v>
+        <v>1.1685</v>
       </c>
     </row>
     <row r="14" ht="12" customHeight="1">
@@ -4263,7 +4293,7 @@
         </is>
       </c>
       <c r="C14" s="24" t="n">
-        <v>0.87253</v>
+        <v>0.87053</v>
       </c>
     </row>
     <row r="15" ht="12" customHeight="1">
@@ -4278,7 +4308,7 @@
         </is>
       </c>
       <c r="C15" s="24" t="n">
-        <v>1.1525</v>
+        <v>1.1685</v>
       </c>
     </row>
     <row r="16" ht="12" customHeight="1">
@@ -4293,7 +4323,7 @@
         </is>
       </c>
       <c r="C16" s="24" t="n">
-        <v>0.87253</v>
+        <v>0.87053</v>
       </c>
     </row>
     <row r="17" ht="12" customHeight="1">
@@ -4308,7 +4338,7 @@
         </is>
       </c>
       <c r="C17" s="24" t="n">
-        <v>1.1525</v>
+        <v>1.1685</v>
       </c>
     </row>
     <row r="18" ht="12" customHeight="1">
@@ -4323,7 +4353,7 @@
         </is>
       </c>
       <c r="C18" s="24" t="n">
-        <v>0.87253</v>
+        <v>0.87053</v>
       </c>
     </row>
     <row r="19" ht="12" customHeight="1">
@@ -4338,7 +4368,7 @@
         </is>
       </c>
       <c r="C19" s="24" t="n">
-        <v>1.1525</v>
+        <v>1.1685</v>
       </c>
     </row>
     <row r="20" ht="12" customHeight="1">
@@ -4353,7 +4383,7 @@
         </is>
       </c>
       <c r="C20" s="24" t="n">
-        <v>0.87253</v>
+        <v>0.87053</v>
       </c>
     </row>
     <row r="21" ht="12" customHeight="1">
@@ -4368,7 +4398,7 @@
         </is>
       </c>
       <c r="C21" s="24" t="n">
-        <v>1.1525</v>
+        <v>1.1685</v>
       </c>
     </row>
     <row r="22" ht="12" customHeight="1">
@@ -4383,7 +4413,7 @@
         </is>
       </c>
       <c r="C22" s="24" t="n">
-        <v>0.87253</v>
+        <v>0.87053</v>
       </c>
     </row>
     <row r="23" ht="12" customHeight="1">
@@ -4398,7 +4428,7 @@
         </is>
       </c>
       <c r="C23" s="24" t="n">
-        <v>1.1525</v>
+        <v>1.1685</v>
       </c>
     </row>
     <row r="24" ht="12" customHeight="1">
@@ -4413,7 +4443,7 @@
         </is>
       </c>
       <c r="C24" s="24" t="n">
-        <v>0.87253</v>
+        <v>0.87053</v>
       </c>
     </row>
     <row r="25" ht="12" customHeight="1">
@@ -4428,7 +4458,7 @@
         </is>
       </c>
       <c r="C25" s="24" t="n">
-        <v>1.1525</v>
+        <v>1.1685</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Adeplus invoice parser
</commit_message>
<xml_diff>
--- a/output/spreadsheet/pyg_consolidado_2026.xlsx
+++ b/output/spreadsheet/pyg_consolidado_2026.xlsx
@@ -712,7 +712,7 @@
     <row r="3" ht="12" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Actualizado: 10/04/2026 11:48 h</t>
+          <t>Actualizado: 10/04/2026 12:53 h</t>
         </is>
       </c>
     </row>
@@ -2625,7 +2625,7 @@
         </is>
       </c>
       <c r="C18" s="23" t="n">
-        <v>2503</v>
+        <v>2812.02</v>
       </c>
     </row>
     <row r="19" ht="12" customHeight="1">
@@ -3045,7 +3045,7 @@
         </is>
       </c>
       <c r="C46" s="23" t="n">
-        <v>54823.58</v>
+        <v>55325.41</v>
       </c>
     </row>
     <row r="47" ht="12" customHeight="1">

</xml_diff>